<commit_message>
feat: Add a Helgeson-Birnie positional weight calculator and line balancing web application.
</commit_message>
<xml_diff>
--- a/Forecast.xlsx
+++ b/Forecast.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr hidePivotFieldList="1" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\Product\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\Product_AMI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9D29501-F06F-42F7-97A3-8DEE5A04E937}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FED2B6A0-C120-4437-ADE4-56EBE3620D24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" firstSheet="4" activeTab="5" xr2:uid="{AC41E7B0-7B6E-4E7F-A6E7-C7838CC9F81E}"/>
   </bookViews>
@@ -317,16 +317,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="187" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="centerContinuous"/>
     </xf>
   </cellXfs>
@@ -4099,10 +4098,10 @@
       <c r="C4">
         <v>41</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="D4" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="E4" s="6"/>
+      <c r="E4" s="5"/>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5">
@@ -4114,10 +4113,10 @@
       <c r="C5">
         <v>37</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" t="s">
         <v>26</v>
       </c>
-      <c r="E5" s="3">
+      <c r="E5">
         <v>0.89630388476297251</v>
       </c>
     </row>
@@ -4131,10 +4130,10 @@
       <c r="C6">
         <v>45</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D6" t="s">
         <v>27</v>
       </c>
-      <c r="E6" s="3">
+      <c r="E6">
         <v>0.80336065384119582</v>
       </c>
     </row>
@@ -4148,10 +4147,10 @@
       <c r="C7">
         <v>50</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="D7" t="s">
         <v>28</v>
       </c>
-      <c r="E7" s="3">
+      <c r="E7">
         <v>0.78369671922531536</v>
       </c>
     </row>
@@ -4165,10 +4164,10 @@
       <c r="C8">
         <v>43</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="D8" t="s">
         <v>29</v>
       </c>
-      <c r="E8" s="3">
+      <c r="E8">
         <v>3.2249934496960999</v>
       </c>
     </row>
@@ -4182,10 +4181,10 @@
       <c r="C9">
         <v>47</v>
       </c>
-      <c r="D9" s="4" t="s">
+      <c r="D9" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="E9" s="4">
+      <c r="E9" s="3">
         <v>12</v>
       </c>
     </row>
@@ -4224,20 +4223,20 @@
       <c r="C12">
         <v>55</v>
       </c>
-      <c r="D12" s="5"/>
-      <c r="E12" s="5" t="s">
+      <c r="D12" s="4"/>
+      <c r="E12" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="F12" s="5" t="s">
+      <c r="F12" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="G12" s="5" t="s">
+      <c r="G12" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="H12" s="5" t="s">
+      <c r="H12" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="I12" s="5" t="s">
+      <c r="I12" s="4" t="s">
         <v>40</v>
       </c>
     </row>
@@ -4251,22 +4250,22 @@
       <c r="C13">
         <v>54</v>
       </c>
-      <c r="D13" s="3" t="s">
+      <c r="D13" t="s">
         <v>32</v>
       </c>
-      <c r="E13" s="3">
+      <c r="E13">
         <v>1</v>
       </c>
-      <c r="F13" s="3">
+      <c r="F13">
         <v>424.91083916083915</v>
       </c>
-      <c r="G13" s="3">
+      <c r="G13">
         <v>424.91083916083915</v>
       </c>
-      <c r="H13" s="3">
+      <c r="H13">
         <v>40.85452222732723</v>
       </c>
-      <c r="I13" s="3">
+      <c r="I13">
         <v>7.9156792254646367E-5</v>
       </c>
     </row>
@@ -4280,118 +4279,116 @@
       <c r="C14" t="s">
         <v>12</v>
       </c>
-      <c r="D14" s="3" t="s">
+      <c r="D14" t="s">
         <v>33</v>
       </c>
-      <c r="E14" s="3">
+      <c r="E14">
         <v>10</v>
       </c>
-      <c r="F14" s="3">
+      <c r="F14">
         <v>104.0058275058275</v>
       </c>
-      <c r="G14" s="3">
+      <c r="G14">
         <v>10.40058275058275</v>
       </c>
-      <c r="H14" s="3"/>
-      <c r="I14" s="3"/>
     </row>
     <row r="15" spans="1:9" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="D15" s="4" t="s">
+      <c r="D15" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="E15" s="4">
+      <c r="E15" s="3">
         <v>11</v>
       </c>
-      <c r="F15" s="4">
+      <c r="F15" s="3">
         <v>528.91666666666663</v>
       </c>
-      <c r="G15" s="4"/>
-      <c r="H15" s="4"/>
-      <c r="I15" s="4"/>
+      <c r="G15" s="3"/>
+      <c r="H15" s="3"/>
+      <c r="I15" s="3"/>
     </row>
     <row r="16" spans="1:9" ht="14.4" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="17" spans="4:12" x14ac:dyDescent="0.25">
-      <c r="D17" s="5"/>
-      <c r="E17" s="5" t="s">
+      <c r="D17" s="4"/>
+      <c r="E17" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="F17" s="5" t="s">
+      <c r="F17" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="G17" s="5" t="s">
+      <c r="G17" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="H17" s="5" t="s">
+      <c r="H17" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="I17" s="5" t="s">
+      <c r="I17" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="J17" s="5" t="s">
+      <c r="J17" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="K17" s="5" t="s">
+      <c r="K17" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="L17" s="5" t="s">
+      <c r="L17" s="4" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="18" spans="4:12" x14ac:dyDescent="0.25">
-      <c r="D18" s="3" t="s">
+      <c r="D18" t="s">
         <v>35</v>
       </c>
-      <c r="E18" s="3">
+      <c r="E18">
         <v>35.212121212121211</v>
       </c>
-      <c r="F18" s="3">
+      <c r="F18">
         <v>1.9848462606083732</v>
       </c>
-      <c r="G18" s="3">
+      <c r="G18">
         <v>17.740477895415626</v>
       </c>
-      <c r="H18" s="3">
+      <c r="H18">
         <v>6.9051559695340924E-9</v>
       </c>
-      <c r="I18" s="3">
+      <c r="I18">
         <v>30.78960814364002</v>
       </c>
-      <c r="J18" s="3">
+      <c r="J18">
         <v>39.634634280602398</v>
       </c>
-      <c r="K18" s="3">
+      <c r="K18">
         <v>30.78960814364002</v>
       </c>
-      <c r="L18" s="3">
+      <c r="L18">
         <v>39.634634280602398</v>
       </c>
     </row>
     <row r="19" spans="4:12" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="D19" s="4" t="s">
+      <c r="D19" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="E19" s="4">
+      <c r="E19" s="3">
         <v>1.7237762237762237</v>
       </c>
-      <c r="F19" s="4">
+      <c r="F19" s="3">
         <v>0.26968750046335682</v>
       </c>
-      <c r="G19" s="4">
+      <c r="G19" s="3">
         <v>6.3917542370875955</v>
       </c>
-      <c r="H19" s="4">
+      <c r="H19" s="3">
         <v>7.9156792254646367E-5</v>
       </c>
-      <c r="I19" s="4">
+      <c r="I19" s="3">
         <v>1.1228750260987521</v>
       </c>
-      <c r="J19" s="4">
+      <c r="J19" s="3">
         <v>2.3246774214536954</v>
       </c>
-      <c r="K19" s="4">
+      <c r="K19" s="3">
         <v>1.1228750260987521</v>
       </c>
-      <c r="L19" s="4">
+      <c r="L19" s="3">
         <v>2.3246774214536954</v>
       </c>
     </row>
@@ -4402,145 +4399,145 @@
     </row>
     <row r="24" spans="4:12" ht="14.4" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="25" spans="4:12" x14ac:dyDescent="0.25">
-      <c r="D25" s="5" t="s">
+      <c r="D25" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="E25" s="5" t="s">
+      <c r="E25" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="F25" s="5" t="s">
+      <c r="F25" s="4" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="26" spans="4:12" x14ac:dyDescent="0.25">
-      <c r="D26" s="3">
+      <c r="D26">
         <v>1</v>
       </c>
-      <c r="E26" s="3">
+      <c r="E26">
         <v>36.935897435897438</v>
       </c>
-      <c r="F26" s="3">
+      <c r="F26">
         <v>6.4102564102562098E-2</v>
       </c>
     </row>
     <row r="27" spans="4:12" x14ac:dyDescent="0.25">
-      <c r="D27" s="3">
+      <c r="D27">
         <v>2</v>
       </c>
-      <c r="E27" s="3">
+      <c r="E27">
         <v>38.659673659673658</v>
       </c>
-      <c r="F27" s="3">
+      <c r="F27">
         <v>1.3403263403263423</v>
       </c>
     </row>
     <row r="28" spans="4:12" x14ac:dyDescent="0.25">
-      <c r="D28" s="3">
+      <c r="D28">
         <v>3</v>
       </c>
-      <c r="E28" s="3">
+      <c r="E28">
         <v>40.383449883449885</v>
       </c>
-      <c r="F28" s="3">
+      <c r="F28">
         <v>0.61655011655011549</v>
       </c>
     </row>
     <row r="29" spans="4:12" x14ac:dyDescent="0.25">
-      <c r="D29" s="3">
+      <c r="D29">
         <v>4</v>
       </c>
-      <c r="E29" s="3">
+      <c r="E29">
         <v>42.107226107226104</v>
       </c>
-      <c r="F29" s="3">
+      <c r="F29">
         <v>-5.1072261072261043</v>
       </c>
     </row>
     <row r="30" spans="4:12" x14ac:dyDescent="0.25">
-      <c r="D30" s="3">
+      <c r="D30">
         <v>5</v>
       </c>
-      <c r="E30" s="3">
+      <c r="E30">
         <v>43.831002331002331</v>
       </c>
-      <c r="F30" s="3">
+      <c r="F30">
         <v>1.1689976689976689</v>
       </c>
     </row>
     <row r="31" spans="4:12" x14ac:dyDescent="0.25">
-      <c r="D31" s="3">
+      <c r="D31">
         <v>6</v>
       </c>
-      <c r="E31" s="3">
+      <c r="E31">
         <v>45.554778554778551</v>
       </c>
-      <c r="F31" s="3">
+      <c r="F31">
         <v>4.4452214452214491</v>
       </c>
     </row>
     <row r="32" spans="4:12" x14ac:dyDescent="0.25">
-      <c r="D32" s="3">
+      <c r="D32">
         <v>7</v>
       </c>
-      <c r="E32" s="3">
+      <c r="E32">
         <v>47.278554778554778</v>
       </c>
-      <c r="F32" s="3">
+      <c r="F32">
         <v>-4.2785547785547777</v>
       </c>
     </row>
     <row r="33" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="D33" s="3">
+      <c r="D33">
         <v>8</v>
       </c>
-      <c r="E33" s="3">
+      <c r="E33">
         <v>49.002331002331005</v>
       </c>
-      <c r="F33" s="3">
+      <c r="F33">
         <v>-2.0023310023310046</v>
       </c>
     </row>
     <row r="34" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="D34" s="3">
+      <c r="D34">
         <v>9</v>
       </c>
-      <c r="E34" s="3">
+      <c r="E34">
         <v>50.726107226107224</v>
       </c>
-      <c r="F34" s="3">
+      <c r="F34">
         <v>5.2738927738927757</v>
       </c>
     </row>
     <row r="35" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="D35" s="3">
+      <c r="D35">
         <v>10</v>
       </c>
-      <c r="E35" s="3">
+      <c r="E35">
         <v>52.449883449883444</v>
       </c>
-      <c r="F35" s="3">
+      <c r="F35">
         <v>-0.44988344988344409</v>
       </c>
     </row>
     <row r="36" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="D36" s="3">
+      <c r="D36">
         <v>11</v>
       </c>
-      <c r="E36" s="3">
+      <c r="E36">
         <v>54.173659673659671</v>
       </c>
-      <c r="F36" s="3">
+      <c r="F36">
         <v>0.82634032634032906</v>
       </c>
     </row>
     <row r="37" spans="4:6" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="D37" s="4">
+      <c r="D37" s="3">
         <v>12</v>
       </c>
-      <c r="E37" s="4">
+      <c r="E37" s="3">
         <v>55.897435897435898</v>
       </c>
-      <c r="F37" s="4">
+      <c r="F37" s="3">
         <v>-1.8974358974358978</v>
       </c>
     </row>
@@ -4623,7 +4620,7 @@
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="B3" s="3">
+      <c r="B3">
         <v>36.935897435897438</v>
       </c>
       <c r="C3">
@@ -4674,7 +4671,7 @@
       <c r="A4">
         <v>37</v>
       </c>
-      <c r="B4" s="3">
+      <c r="B4">
         <v>38.659673659673658</v>
       </c>
       <c r="C4">
@@ -4723,7 +4720,7 @@
         <v>-1</v>
       </c>
       <c r="O4">
-        <f>G4/K4</f>
+        <f t="shared" ref="O4:O14" si="2">G4/K4</f>
         <v>2</v>
       </c>
     </row>
@@ -4731,14 +4728,14 @@
       <c r="A5">
         <v>37.9</v>
       </c>
-      <c r="B5" s="3">
+      <c r="B5">
         <v>40.383449883449885</v>
       </c>
       <c r="C5">
         <v>41</v>
       </c>
       <c r="D5">
-        <f t="shared" ref="D5:D15" si="2">ABS(C5-A5)</f>
+        <f t="shared" ref="D5:D15" si="3">ABS(C5-A5)</f>
         <v>3.1000000000000014</v>
       </c>
       <c r="E5">
@@ -4746,11 +4743,11 @@
         <v>0.61655011655011549</v>
       </c>
       <c r="F5">
-        <f t="shared" ref="F5:F15" si="3">F4+D5</f>
+        <f t="shared" ref="F5:F15" si="4">F4+D5</f>
         <v>6.1000000000000014</v>
       </c>
       <c r="G5">
-        <f t="shared" ref="G5:G15" si="4">G4+E5</f>
+        <f t="shared" ref="G5:G15" si="5">G4+E5</f>
         <v>2.0209790209790199</v>
       </c>
       <c r="H5">
@@ -4760,7 +4757,7 @@
         <v>3</v>
       </c>
       <c r="J5">
-        <f t="shared" ref="J5:J14" si="5">F5/H5</f>
+        <f t="shared" ref="J5:J14" si="6">F5/H5</f>
         <v>3.0500000000000007</v>
       </c>
       <c r="K5">
@@ -4768,19 +4765,19 @@
         <v>0.67365967365967327</v>
       </c>
       <c r="L5">
-        <f t="shared" ref="L5:L15" si="6">(C5-A5)</f>
+        <f t="shared" ref="L5:L15" si="7">(C5-A5)</f>
         <v>3.1000000000000014</v>
       </c>
       <c r="M5">
-        <f t="shared" ref="L5:M15" si="7">(C5-B5)+M4</f>
+        <f t="shared" ref="M5:M15" si="8">(C5-B5)+M4</f>
         <v>2.0209790209790199</v>
       </c>
       <c r="N5">
-        <f t="shared" ref="N5:N15" si="8">-F5/J5</f>
+        <f t="shared" ref="N5:N15" si="9">-F5/J5</f>
         <v>-2</v>
       </c>
       <c r="O5">
-        <f>G5/K5</f>
+        <f t="shared" si="2"/>
         <v>3</v>
       </c>
     </row>
@@ -4788,14 +4785,14 @@
       <c r="A6">
         <v>38.83</v>
       </c>
-      <c r="B6" s="3">
+      <c r="B6">
         <v>42.107226107226104</v>
       </c>
       <c r="C6">
         <v>37</v>
       </c>
       <c r="D6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1.8299999999999983</v>
       </c>
       <c r="E6">
@@ -4803,11 +4800,11 @@
         <v>5.1072261072261043</v>
       </c>
       <c r="F6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>7.93</v>
       </c>
       <c r="G6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>7.1282051282051242</v>
       </c>
       <c r="H6">
@@ -4817,7 +4814,7 @@
         <v>4</v>
       </c>
       <c r="J6">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>2.6433333333333331</v>
       </c>
       <c r="K6">
@@ -4825,19 +4822,19 @@
         <v>1.782051282051281</v>
       </c>
       <c r="L6">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>-1.8299999999999983</v>
       </c>
       <c r="M6">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>-3.0862470862470843</v>
       </c>
       <c r="N6">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>-3</v>
       </c>
       <c r="O6">
-        <f>G6/K6</f>
+        <f t="shared" si="2"/>
         <v>4</v>
       </c>
     </row>
@@ -4845,14 +4842,14 @@
       <c r="A7">
         <v>38.280999999999999</v>
       </c>
-      <c r="B7" s="3">
+      <c r="B7">
         <v>43.831002331002331</v>
       </c>
       <c r="C7">
         <v>45</v>
       </c>
       <c r="D7">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>6.7190000000000012</v>
       </c>
       <c r="E7">
@@ -4860,11 +4857,11 @@
         <v>1.1689976689976689</v>
       </c>
       <c r="F7">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>14.649000000000001</v>
       </c>
       <c r="G7">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>8.2972027972027931</v>
       </c>
       <c r="H7">
@@ -4874,7 +4871,7 @@
         <v>5</v>
       </c>
       <c r="J7">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>3.6622500000000002</v>
       </c>
       <c r="K7">
@@ -4882,19 +4879,19 @@
         <v>1.6594405594405586</v>
       </c>
       <c r="L7">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>6.7190000000000012</v>
       </c>
       <c r="M7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>-1.9172494172494154</v>
       </c>
       <c r="N7">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>-4</v>
       </c>
       <c r="O7">
-        <f>G7/K7</f>
+        <f t="shared" si="2"/>
         <v>5</v>
       </c>
     </row>
@@ -4902,14 +4899,14 @@
       <c r="A8">
         <v>40.296700000000001</v>
       </c>
-      <c r="B8" s="3">
+      <c r="B8">
         <v>45.554778554778551</v>
       </c>
       <c r="C8">
         <v>50</v>
       </c>
       <c r="D8">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>9.7032999999999987</v>
       </c>
       <c r="E8">
@@ -4917,11 +4914,11 @@
         <v>4.4452214452214491</v>
       </c>
       <c r="F8">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>24.3523</v>
       </c>
       <c r="G8">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>12.742424242424242</v>
       </c>
       <c r="H8">
@@ -4931,7 +4928,7 @@
         <v>6</v>
       </c>
       <c r="J8">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>4.8704599999999996</v>
       </c>
       <c r="K8">
@@ -4939,19 +4936,19 @@
         <v>2.1237373737373737</v>
       </c>
       <c r="L8">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>9.7032999999999987</v>
       </c>
       <c r="M8">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>2.5279720279720337</v>
       </c>
       <c r="N8">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>-5</v>
       </c>
       <c r="O8">
-        <f>G8/K8</f>
+        <f t="shared" si="2"/>
         <v>6</v>
       </c>
     </row>
@@ -4959,14 +4956,14 @@
       <c r="A9">
         <v>43.207689999999999</v>
       </c>
-      <c r="B9" s="3">
+      <c r="B9">
         <v>47.278554778554778</v>
       </c>
       <c r="C9">
         <v>43</v>
       </c>
       <c r="D9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.20768999999999949</v>
       </c>
       <c r="E9">
@@ -4974,11 +4971,11 @@
         <v>4.2785547785547777</v>
       </c>
       <c r="F9">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>24.559989999999999</v>
       </c>
       <c r="G9">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>17.02097902097902</v>
       </c>
       <c r="H9">
@@ -4988,7 +4985,7 @@
         <v>7</v>
       </c>
       <c r="J9">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>4.0933316666666668</v>
       </c>
       <c r="K9">
@@ -4996,19 +4993,19 @@
         <v>2.4315684315684316</v>
       </c>
       <c r="L9">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>-0.20768999999999949</v>
       </c>
       <c r="M9">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>-1.750582750582744</v>
       </c>
       <c r="N9">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>-6</v>
       </c>
       <c r="O9">
-        <f>G9/K9</f>
+        <f t="shared" si="2"/>
         <v>6.9999999999999991</v>
       </c>
     </row>
@@ -5016,14 +5013,14 @@
       <c r="A10">
         <v>43.145382999999995</v>
       </c>
-      <c r="B10" s="3">
+      <c r="B10">
         <v>49.002331002331005</v>
       </c>
       <c r="C10">
         <v>47</v>
       </c>
       <c r="D10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>3.8546170000000046</v>
       </c>
       <c r="E10">
@@ -5031,11 +5028,11 @@
         <v>2.0023310023310046</v>
       </c>
       <c r="F10">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>28.414607000000004</v>
       </c>
       <c r="G10">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>19.023310023310025</v>
       </c>
       <c r="H10">
@@ -5045,7 +5042,7 @@
         <v>8</v>
       </c>
       <c r="J10">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>4.0592295714285722</v>
       </c>
       <c r="K10">
@@ -5053,19 +5050,19 @@
         <v>2.3779137529137531</v>
       </c>
       <c r="L10">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>3.8546170000000046</v>
       </c>
       <c r="M10">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>-3.7529137529137486</v>
       </c>
       <c r="N10">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>-7</v>
       </c>
       <c r="O10">
-        <f>G10/K10</f>
+        <f t="shared" si="2"/>
         <v>8</v>
       </c>
     </row>
@@ -5073,14 +5070,14 @@
       <c r="A11">
         <v>44.301768099999997</v>
       </c>
-      <c r="B11" s="3">
+      <c r="B11">
         <v>50.726107226107224</v>
       </c>
       <c r="C11">
         <v>56</v>
       </c>
       <c r="D11">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>11.698231900000003</v>
       </c>
       <c r="E11">
@@ -5088,11 +5085,11 @@
         <v>5.2738927738927757</v>
       </c>
       <c r="F11">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>40.112838900000007</v>
       </c>
       <c r="G11">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>24.2972027972028</v>
       </c>
       <c r="H11">
@@ -5102,7 +5099,7 @@
         <v>9</v>
       </c>
       <c r="J11">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>5.0141048625000009</v>
       </c>
       <c r="K11">
@@ -5110,19 +5107,19 @@
         <v>2.6996891996892001</v>
       </c>
       <c r="L11">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>11.698231900000003</v>
       </c>
       <c r="M11">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>1.520979020979027</v>
       </c>
       <c r="N11">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>-8</v>
       </c>
       <c r="O11">
-        <f>G11/K11</f>
+        <f t="shared" si="2"/>
         <v>9</v>
       </c>
     </row>
@@ -5130,14 +5127,14 @@
       <c r="A12">
         <v>47.811237669999997</v>
       </c>
-      <c r="B12" s="3">
+      <c r="B12">
         <v>52.449883449883444</v>
       </c>
       <c r="C12">
         <v>52</v>
       </c>
       <c r="D12">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>4.188762330000003</v>
       </c>
       <c r="E12">
@@ -5145,11 +5142,11 @@
         <v>0.44988344988344409</v>
       </c>
       <c r="F12">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>44.30160123000001</v>
       </c>
       <c r="G12">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>24.747086247086244</v>
       </c>
       <c r="H12">
@@ -5159,7 +5156,7 @@
         <v>10</v>
       </c>
       <c r="J12">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>4.9224001366666679</v>
       </c>
       <c r="K12">
@@ -5167,19 +5164,19 @@
         <v>2.4747086247086245</v>
       </c>
       <c r="L12">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>4.188762330000003</v>
       </c>
       <c r="M12">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>1.071095571095583</v>
       </c>
       <c r="N12">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>-9</v>
       </c>
       <c r="O12">
-        <f>G12/K12</f>
+        <f t="shared" si="2"/>
         <v>10</v>
       </c>
     </row>
@@ -5187,14 +5184,14 @@
       <c r="A13">
         <v>49.067866369000001</v>
       </c>
-      <c r="B13" s="3">
+      <c r="B13">
         <v>54.173659673659671</v>
       </c>
       <c r="C13">
         <v>55</v>
       </c>
       <c r="D13">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>5.9321336309999992</v>
       </c>
       <c r="E13">
@@ -5202,11 +5199,11 @@
         <v>0.82634032634032906</v>
       </c>
       <c r="F13">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>50.233734861000009</v>
       </c>
       <c r="G13">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>25.573426573426573</v>
       </c>
       <c r="H13">
@@ -5216,7 +5213,7 @@
         <v>11</v>
       </c>
       <c r="J13">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>5.0233734861000006</v>
       </c>
       <c r="K13">
@@ -5224,19 +5221,19 @@
         <v>2.3248569612205974</v>
       </c>
       <c r="L13">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>5.9321336309999992</v>
       </c>
       <c r="M13">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>1.897435897435912</v>
       </c>
       <c r="N13">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>-10</v>
       </c>
       <c r="O13">
-        <f>G13/K13</f>
+        <f t="shared" si="2"/>
         <v>11.000000000000002</v>
       </c>
     </row>
@@ -5244,14 +5241,14 @@
       <c r="A14">
         <v>50.847506458299996</v>
       </c>
-      <c r="B14" s="4">
+      <c r="B14" s="3">
         <v>55.897435897435898</v>
       </c>
       <c r="C14">
         <v>54</v>
       </c>
       <c r="D14">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>3.1524935417000037</v>
       </c>
       <c r="E14">
@@ -5259,11 +5256,11 @@
         <v>1.8974358974358978</v>
       </c>
       <c r="F14">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>53.386228402700013</v>
       </c>
       <c r="G14">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>27.470862470862471</v>
       </c>
       <c r="H14">
@@ -5273,7 +5270,7 @@
         <v>12</v>
       </c>
       <c r="J14">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>4.8532934911545462</v>
       </c>
       <c r="K14">
@@ -5281,19 +5278,19 @@
         <v>2.2892385392385393</v>
       </c>
       <c r="L14">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>3.1524935417000037</v>
       </c>
       <c r="M14">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>1.4210854715202004E-14</v>
       </c>
       <c r="N14">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>-11.000000000000002</v>
       </c>
       <c r="O14">
-        <f>G14/K14</f>
+        <f t="shared" si="2"/>
         <v>12</v>
       </c>
     </row>
@@ -5306,7 +5303,7 @@
         <v>57.56</v>
       </c>
       <c r="D15">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>51.793254520809995</v>
       </c>
       <c r="E15">
@@ -5314,23 +5311,23 @@
         <v>57.56</v>
       </c>
       <c r="F15">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>105.17948292351001</v>
       </c>
       <c r="G15">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>85.030862470862473</v>
       </c>
       <c r="L15">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>-51.793254520809995</v>
       </c>
       <c r="M15">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>-57.559999999999988</v>
       </c>
       <c r="N15" t="e">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>#DIV/0!</v>
       </c>
     </row>

</xml_diff>